<commit_message>
Dashboard refresh 2026-06-06 12:35
</commit_message>
<xml_diff>
--- a/streamlit_data/price_alerts.xlsx
+++ b/streamlit_data/price_alerts.xlsx
@@ -1406,34 +1406,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>festival_noel festival chocolate_unknown</t>
+          <t>confetti_confetti mini gelatinas_unknown</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Festival</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>NOEL FESTIVAL CHOCOLATE</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.3365384615384615</v>
+        <v>2.788461538461538</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Festival</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NOEL FESTIVAL CHOCOLATE</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>3.942307692307693</v>
+        <v>1.394230769230769</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>-91.46341463414633</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
@@ -1457,34 +1457,34 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>festival_noel festival chocolate_unknown</t>
+          <t>confetti_confetti mini gelatinas_unknown</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Festival</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>NOEL FESTIVAL CHOCOLATE</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.942307692307693</v>
+        <v>2.788461538461538</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Festival</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>NOEL FESTIVAL CHOCOLATE</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>0.3365384615384615</v>
+        <v>0.7211538461538461</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>1071.428571428572</v>
+        <v>286.6666666666666</v>
       </c>
     </row>
     <row r="22">
@@ -1508,34 +1508,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>instorebakery_holiday cheeze puffs_unknown</t>
+          <t>confetti_confetti mini gelatinas_unknown</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Instorebakery</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Holiday Cheeze Puffs</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1.730769230769231</v>
+        <v>1.394230769230769</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Instorebakery</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Holiday Cheeze Puffs</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>0.4326923076923077</v>
+        <v>2.788461538461538</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>300</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="23">
@@ -1559,34 +1559,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>instorebakery_holiday cheeze puffs_unknown</t>
+          <t>confetti_confetti mini gelatinas_unknown</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Instorebakery</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Holiday Cheeze Puffs</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>0.4326923076923077</v>
+        <v>1.394230769230769</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Instorebakery</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Holiday Cheeze Puffs</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>1.730769230769231</v>
+        <v>0.7211538461538461</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>-75</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
     <row r="24">
@@ -1610,34 +1610,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>kugi_kugi chocolate wafer sticks_unknown</t>
+          <t>confetti_confetti mini gelatinas_unknown</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>KUGI CHOCOLATE WAFER STICKS</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1.682692307692308</v>
+        <v>0.7211538461538461</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Kugi Chocolate Wafer Sticks</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>4.086538461538462</v>
+        <v>2.788461538461538</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1645,7 +1645,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>-58.82352941176471</v>
+        <v>-74.13793103448275</v>
       </c>
     </row>
     <row r="25">
@@ -1661,34 +1661,34 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>kugi_kugi chocolate wafer sticks_unknown</t>
+          <t>confetti_confetti mini gelatinas_unknown</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Kugi Chocolate Wafer Sticks</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>4.086538461538462</v>
+        <v>0.7211538461538461</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Confetti</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>KUGI CHOCOLATE WAFER STICKS</t>
+          <t>Confetti Mini Gelatinas</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>1.682692307692308</v>
+        <v>1.394230769230769</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>142.8571428571429</v>
+        <v>-48.27586206896552</v>
       </c>
     </row>
     <row r="26">
@@ -1712,34 +1712,34 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>kugi_kugi vanilla milk wafer sticks_unknown</t>
+          <t>festival_noel festival chocolate_unknown</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Festival</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>KUGI VANILLA MILK WAFER STICKS</t>
+          <t>NOEL FESTIVAL CHOCOLATE</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1.682692307692308</v>
+        <v>0.3365384615384615</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Festival</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Kugi Vanilla Milk Wafer Sticks</t>
+          <t>NOEL FESTIVAL CHOCOLATE</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>4.086538461538462</v>
+        <v>3.942307692307693</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1747,7 +1747,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>-58.82352941176471</v>
+        <v>-91.46341463414633</v>
       </c>
     </row>
     <row r="27">
@@ -1763,34 +1763,34 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>kugi_kugi vanilla milk wafer sticks_unknown</t>
+          <t>festival_noel festival chocolate_unknown</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Festival</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Kugi Vanilla Milk Wafer Sticks</t>
+          <t>NOEL FESTIVAL CHOCOLATE</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>4.086538461538462</v>
+        <v>3.942307692307693</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Festival</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>KUGI VANILLA MILK WAFER STICKS</t>
+          <t>NOEL FESTIVAL CHOCOLATE</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>1.682692307692308</v>
+        <v>0.3365384615384615</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -1798,7 +1798,7 @@
         </is>
       </c>
       <c r="K27" t="n">
-        <v>142.8571428571429</v>
+        <v>1071.428571428572</v>
       </c>
     </row>
     <row r="28">
@@ -1814,34 +1814,34 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>oh snacks_oh snacks quinoa_unknown</t>
+          <t>instorebakery_holiday cheeze puffs_unknown</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Oh Snacks</t>
+          <t>Instorebakery</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Oh Snacks Quinoa</t>
+          <t>Holiday Cheeze Puffs</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>5.576923076923077</v>
+        <v>1.730769230769231</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Oh Snacks</t>
+          <t>Instorebakery</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Oh Snacks Quinoa</t>
+          <t>Holiday Cheeze Puffs</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>12.35576923076923</v>
+        <v>0.4326923076923077</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>-54.86381322957198</v>
+        <v>300</v>
       </c>
     </row>
     <row r="29">
@@ -1865,34 +1865,34 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>oh snacks_oh snacks quinoa_unknown</t>
+          <t>instorebakery_holiday cheeze puffs_unknown</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Oh Snacks</t>
+          <t>Instorebakery</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Oh Snacks Quinoa</t>
+          <t>Holiday Cheeze Puffs</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>12.35576923076923</v>
+        <v>0.4326923076923077</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Oh Snacks</t>
+          <t>Instorebakery</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Oh Snacks Quinoa</t>
+          <t>Holiday Cheeze Puffs</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>5.576923076923077</v>
+        <v>1.730769230769231</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>121.551724137931</v>
+        <v>-75</v>
       </c>
     </row>
     <row r="30">
@@ -1916,34 +1916,34 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>other_toppers caramel popcorn_unknown</t>
+          <t>kugi_kugi chocolate wafer sticks_unknown</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Toppers Caramel Popcorn</t>
+          <t>KUGI CHOCOLATE WAFER STICKS</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>4.326923076923077</v>
+        <v>1.682692307692308</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Toppers Caramel Popcorn</t>
+          <t>Kugi Chocolate Wafer Sticks</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>1.057692307692308</v>
+        <v>4.086538461538462</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="K30" t="n">
-        <v>309.0909090909091</v>
+        <v>-58.82352941176471</v>
       </c>
     </row>
     <row r="31">
@@ -1967,34 +1967,34 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>other_toppers caramel popcorn_unknown</t>
+          <t>kugi_kugi chocolate wafer sticks_unknown</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Toppers Caramel Popcorn</t>
+          <t>Kugi Chocolate Wafer Sticks</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1.057692307692308</v>
+        <v>4.086538461538462</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Toppers Caramel Popcorn</t>
+          <t>KUGI CHOCOLATE WAFER STICKS</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>4.326923076923077</v>
+        <v>1.682692307692308</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>-75.55555555555556</v>
+        <v>142.8571428571429</v>
       </c>
     </row>
     <row r="32">
@@ -2018,34 +2018,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>other_toppers frosted popcorn_unknown</t>
+          <t>kugi_kugi vanilla milk wafer sticks_unknown</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Toppers Frosted Popcorn</t>
+          <t>KUGI VANILLA MILK WAFER STICKS</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>4.326923076923077</v>
+        <v>1.682692307692308</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Toppers Frosted Popcorn</t>
+          <t>Kugi Vanilla Milk Wafer Sticks</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>1.105769230769231</v>
+        <v>4.086538461538462</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="K32" t="n">
-        <v>291.3043478260869</v>
+        <v>-58.82352941176471</v>
       </c>
     </row>
     <row r="33">
@@ -2069,34 +2069,34 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>other_toppers frosted popcorn_unknown</t>
+          <t>kugi_kugi vanilla milk wafer sticks_unknown</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Toppers Frosted Popcorn</t>
+          <t>Kugi Vanilla Milk Wafer Sticks</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1.105769230769231</v>
+        <v>4.086538461538462</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Toppers Frosted Popcorn</t>
+          <t>KUGI VANILLA MILK WAFER STICKS</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>4.326923076923077</v>
+        <v>1.682692307692308</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="K33" t="n">
-        <v>-74.44444444444444</v>
+        <v>142.8571428571429</v>
       </c>
     </row>
     <row r="34">
@@ -2120,34 +2120,34 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>other_toppers kettle popcorn_unknown</t>
+          <t>oh snacks_oh snacks quinoa_unknown</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Oh Snacks</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Toppers Kettle Popcorn</t>
+          <t>Oh Snacks Quinoa</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>4.134615384615385</v>
+        <v>5.576923076923077</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Oh Snacks</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Toppers Kettle Popcorn</t>
+          <t>Oh Snacks Quinoa</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>1.057692307692308</v>
+        <v>12.35576923076923</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
       <c r="K34" t="n">
-        <v>290.9090909090909</v>
+        <v>-54.86381322957198</v>
       </c>
     </row>
     <row r="35">
@@ -2171,34 +2171,34 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>other_toppers kettle popcorn_unknown</t>
+          <t>oh snacks_oh snacks quinoa_unknown</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Oh Snacks</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Toppers Kettle Popcorn</t>
+          <t>Oh Snacks Quinoa</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1.057692307692308</v>
+        <v>12.35576923076923</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Oh Snacks</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Toppers Kettle Popcorn</t>
+          <t>Oh Snacks Quinoa</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>4.134615384615385</v>
+        <v>5.576923076923077</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -2206,7 +2206,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>-74.41860465116279</v>
+        <v>121.551724137931</v>
       </c>
     </row>
     <row r="36">
@@ -2222,34 +2222,34 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>pepperidge_pepperidge farm goldfish cheddar_unknown</t>
+          <t>other_toppers caramel popcorn_unknown</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Pepperidge</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>PEPPERIDGE FARM GOLDFISH CHEDDAR</t>
+          <t>Toppers Caramel Popcorn</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1.201923076923077</v>
+        <v>4.326923076923077</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Pepperidge</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Pepperidge Farm Goldfish Cheddar</t>
+          <t>Toppers Caramel Popcorn</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>0.8653846153846154</v>
+        <v>1.057692307692308</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>38.88888888888888</v>
+        <v>309.0909090909091</v>
       </c>
     </row>
     <row r="37">
@@ -2273,34 +2273,34 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>pepperidge_pepperidge farm goldfish cheddar_unknown</t>
+          <t>other_toppers caramel popcorn_unknown</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Pepperidge</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Pepperidge Farm Goldfish Cheddar</t>
+          <t>Toppers Caramel Popcorn</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0.8653846153846154</v>
+        <v>1.057692307692308</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Pepperidge</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>PEPPERIDGE FARM GOLDFISH CHEDDAR</t>
+          <t>Toppers Caramel Popcorn</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>1.201923076923077</v>
+        <v>4.326923076923077</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2308,7 +2308,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>-27.99999999999999</v>
+        <v>-75.55555555555556</v>
       </c>
     </row>
     <row r="38">
@@ -2324,34 +2324,34 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>pringles_pringles pizza_unknown</t>
+          <t>other_toppers frosted popcorn_unknown</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Pringles</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PRINGLES PIZZA</t>
+          <t>Toppers Frosted Popcorn</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.254807692307693</v>
+        <v>4.326923076923077</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Pringles</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Pringles Pizza</t>
+          <t>Toppers Frosted Popcorn</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>2.5</v>
+        <v>1.105769230769231</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -2359,7 +2359,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>70.19230769230769</v>
+        <v>291.3043478260869</v>
       </c>
     </row>
     <row r="39">
@@ -2375,34 +2375,34 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>pringles_pringles pizza_unknown</t>
+          <t>other_toppers frosted popcorn_unknown</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Pringles</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Pringles Pizza</t>
+          <t>Toppers Frosted Popcorn</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2.5</v>
+        <v>1.105769230769231</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Pringles</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>PRINGLES PIZZA</t>
+          <t>Toppers Frosted Popcorn</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>4.254807692307693</v>
+        <v>4.326923076923077</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>-41.24293785310735</v>
+        <v>-74.44444444444444</v>
       </c>
     </row>
     <row r="40">
@@ -2426,34 +2426,34 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>shoon_shoon fatt cream crackers_unknown</t>
+          <t>other_toppers kettle popcorn_unknown</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Shoon</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Shoon Fatt Cream Crackers</t>
+          <t>Toppers Kettle Popcorn</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>10.86538461538462</v>
+        <v>4.134615384615385</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Shoon</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>SHOON FATT CREAM CRACKERS</t>
+          <t>Toppers Kettle Popcorn</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>1.826923076923077</v>
+        <v>1.057692307692308</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2461,7 +2461,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>494.7368421052633</v>
+        <v>290.9090909090909</v>
       </c>
     </row>
     <row r="41">
@@ -2477,34 +2477,34 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>shoon_shoon fatt cream crackers_unknown</t>
+          <t>other_toppers kettle popcorn_unknown</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Shoon</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>SHOON FATT CREAM CRACKERS</t>
+          <t>Toppers Kettle Popcorn</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1.826923076923077</v>
+        <v>1.057692307692308</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Shoon</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Shoon Fatt Cream Crackers</t>
+          <t>Toppers Kettle Popcorn</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>10.86538461538462</v>
+        <v>4.134615384615385</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="K41" t="n">
-        <v>-83.18584070796462</v>
+        <v>-74.41860465116279</v>
       </c>
     </row>
     <row r="42">
@@ -2528,34 +2528,34 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>sunshine snacks_sunshine cashew nuts light salt_unknown</t>
+          <t>pepperidge_pepperidge farm goldfish cheddar_unknown</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Sunshine Snacks</t>
+          <t>Pepperidge</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Sunshine Cashew Nuts Light Salt</t>
+          <t>PEPPERIDGE FARM GOLDFISH CHEDDAR</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>1.778846153846154</v>
+        <v>1.201923076923077</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Sunshine Snacks</t>
+          <t>Pepperidge</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Sunshine Cashew Nuts Light Salt</t>
+          <t>Pepperidge Farm Goldfish Cheddar</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>1.105769230769231</v>
+        <v>0.8653846153846154</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -2563,7 +2563,7 @@
         </is>
       </c>
       <c r="K42" t="n">
-        <v>60.86956521739126</v>
+        <v>38.88888888888888</v>
       </c>
     </row>
     <row r="43">
@@ -2579,34 +2579,34 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>sunshine snacks_sunshine cashew nuts light salt_unknown</t>
+          <t>pepperidge_pepperidge farm goldfish cheddar_unknown</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Sunshine Snacks</t>
+          <t>Pepperidge</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Sunshine Cashew Nuts Light Salt</t>
+          <t>Pepperidge Farm Goldfish Cheddar</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>1.105769230769231</v>
+        <v>0.8653846153846154</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Sunshine Snacks</t>
+          <t>Pepperidge</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Sunshine Cashew Nuts Light Salt</t>
+          <t>PEPPERIDGE FARM GOLDFISH CHEDDAR</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>1.778846153846154</v>
+        <v>1.201923076923077</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -2614,7 +2614,7 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>-37.83783783783782</v>
+        <v>-27.99999999999999</v>
       </c>
     </row>
     <row r="44">
@@ -2630,34 +2630,34 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>triskits_triskits vanilla crackers_unknown</t>
+          <t>pringles_pringles pizza_unknown</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Pringles</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>PRINGLES PIZZA</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1.610576923076923</v>
+        <v>4.254807692307693</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Pringles</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Pringles Pizza</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>1.346153846153846</v>
+        <v>2.5</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="K44" t="n">
-        <v>19.64285714285712</v>
+        <v>70.19230769230769</v>
       </c>
     </row>
     <row r="45">
@@ -2681,34 +2681,34 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>triskits_triskits vanilla crackers_unknown</t>
+          <t>pringles_pringles pizza_unknown</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Pringles</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Pringles Pizza</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1.610576923076923</v>
+        <v>2.5</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Pringles</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>PRINGLES PIZZA</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.5769230769230769</v>
+        <v>4.254807692307693</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -2716,7 +2716,7 @@
         </is>
       </c>
       <c r="K45" t="n">
-        <v>179.1666666666667</v>
+        <v>-41.24293785310735</v>
       </c>
     </row>
     <row r="46">
@@ -2732,34 +2732,34 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>triskits_triskits vanilla crackers_unknown</t>
+          <t>shoon_shoon fatt cream crackers_unknown</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Shoon</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Shoon Fatt Cream Crackers</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1.346153846153846</v>
+        <v>10.86538461538462</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Shoon</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>SHOON FATT CREAM CRACKERS</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>1.610576923076923</v>
+        <v>1.826923076923077</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>-16.41791044776118</v>
+        <v>494.7368421052633</v>
       </c>
     </row>
     <row r="47">
@@ -2783,34 +2783,34 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>triskits_triskits vanilla crackers_unknown</t>
+          <t>shoon_shoon fatt cream crackers_unknown</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Shoon</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>SHOON FATT CREAM CRACKERS</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>1.346153846153846</v>
+        <v>1.826923076923077</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Shoon</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Shoon Fatt Cream Crackers</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>0.5769230769230769</v>
+        <v>10.86538461538462</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -2818,7 +2818,7 @@
         </is>
       </c>
       <c r="K47" t="n">
-        <v>133.3333333333334</v>
+        <v>-83.18584070796462</v>
       </c>
     </row>
     <row r="48">
@@ -2834,34 +2834,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>triskits_triskits vanilla crackers_unknown</t>
+          <t>sunshine snacks_sunshine cashew nuts light salt_unknown</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Sunshine Snacks</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Sunshine Cashew Nuts Light Salt</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>0.5769230769230769</v>
+        <v>1.778846153846154</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Sunshine Snacks</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Sunshine Cashew Nuts Light Salt</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>1.610576923076923</v>
+        <v>1.105769230769231</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>-64.17910447761194</v>
+        <v>60.86956521739126</v>
       </c>
     </row>
     <row r="49">
@@ -2885,34 +2885,34 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>triskits_triskits vanilla crackers_unknown</t>
+          <t>sunshine snacks_sunshine cashew nuts light salt_unknown</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Sunshine Snacks</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Sunshine Cashew Nuts Light Salt</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>0.5769230769230769</v>
+        <v>1.105769230769231</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Sunshine Snacks</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Sunshine Cashew Nuts Light Salt</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>1.346153846153846</v>
+        <v>1.778846153846154</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="K49" t="n">
-        <v>-57.14285714285716</v>
+        <v>-37.83783783783782</v>
       </c>
     </row>
     <row r="50">
@@ -2936,34 +2936,34 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>unknown_confetti mini gelatinas_unknown</t>
+          <t>triskits_triskits vanilla crackers_unknown</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>2.788461538461538</v>
+        <v>1.610576923076923</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>1.394230769230769</v>
+        <v>1.346153846153846</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>100</v>
+        <v>19.64285714285712</v>
       </c>
     </row>
     <row r="51">
@@ -2987,34 +2987,34 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>unknown_confetti mini gelatinas_unknown</t>
+          <t>triskits_triskits vanilla crackers_unknown</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>2.788461538461538</v>
+        <v>1.610576923076923</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>0.7211538461538461</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>286.6666666666666</v>
+        <v>179.1666666666667</v>
       </c>
     </row>
     <row r="52">
@@ -3038,34 +3038,34 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>unknown_confetti mini gelatinas_unknown</t>
+          <t>triskits_triskits vanilla crackers_unknown</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1.394230769230769</v>
+        <v>1.346153846153846</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="I52" t="n">
-        <v>2.788461538461538</v>
+        <v>1.610576923076923</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>-50</v>
+        <v>-16.41791044776118</v>
       </c>
     </row>
     <row r="53">
@@ -3089,34 +3089,34 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>unknown_confetti mini gelatinas_unknown</t>
+          <t>triskits_triskits vanilla crackers_unknown</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>1.394230769230769</v>
+        <v>1.346153846153846</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="I53" t="n">
-        <v>0.7211538461538461</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3124,7 +3124,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>93.33333333333333</v>
+        <v>133.3333333333334</v>
       </c>
     </row>
     <row r="54">
@@ -3140,34 +3140,34 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>unknown_confetti mini gelatinas_unknown</t>
+          <t>triskits_triskits vanilla crackers_unknown</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>0.7211538461538461</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="I54" t="n">
-        <v>2.788461538461538</v>
+        <v>1.610576923076923</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>-74.13793103448275</v>
+        <v>-64.17910447761194</v>
       </c>
     </row>
     <row r="55">
@@ -3191,34 +3191,34 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>unknown_confetti mini gelatinas_unknown</t>
+          <t>triskits_triskits vanilla crackers_unknown</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>0.7211538461538461</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Confetti Mini Gelatinas</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>1.394230769230769</v>
+        <v>1.346153846153846</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -3226,7 +3226,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>-48.27586206896552</v>
+        <v>-57.14285714285716</v>
       </c>
     </row>
     <row r="56">
@@ -3342,7 +3342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3401,45 +3401,6 @@
           <t>price_change_pct</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>post_mezcla reposteria duncan hines bizcocho fresa_0.43</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Post</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Mezcla Reposteria Duncan Hines Bizcocho Fresa</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3452,7 +3413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3512,45 +3473,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>unknown_mezcla reposteria duncan hines bizcocho fresa_0.43</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Mezcla Reposteria Duncan Hines Bizcocho Fresa</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Filter fake category rows from regional master
</commit_message>
<xml_diff>
--- a/streamlit_data/price_alerts.xlsx
+++ b/streamlit_data/price_alerts.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>shoon_shoon fatt cream crackers_unknown</t>
+          <t>shoon_shoon fatt butter crackers_unknown</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2742,11 +2742,11 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Shoon Fatt Cream Crackers</t>
+          <t>SHOON FATT BUTTER CRACKERS</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>10.86538461538462</v>
+        <v>1.778846153846154</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2755,11 +2755,11 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>SHOON FATT CREAM CRACKERS</t>
+          <t>Shoon Fatt Butter Crackers</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>1.826923076923077</v>
+        <v>4.182692307692307</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -2767,7 +2767,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>494.7368421052633</v>
+        <v>-57.4712643678161</v>
       </c>
     </row>
     <row r="47">
@@ -2793,32 +2793,32 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
+          <t>Shoon Fatt Cream Crackers</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>10.86538461538462</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Shoon</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
           <t>SHOON FATT CREAM CRACKERS</t>
         </is>
       </c>
-      <c r="F47" t="n">
+      <c r="I47" t="n">
         <v>1.826923076923077</v>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Shoon</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Shoon Fatt Cream Crackers</t>
-        </is>
-      </c>
-      <c r="I47" t="n">
-        <v>10.86538461538462</v>
-      </c>
       <c r="J47" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
       <c r="K47" t="n">
-        <v>-83.18584070796462</v>
+        <v>494.7368421052633</v>
       </c>
     </row>
     <row r="48">
@@ -2834,34 +2834,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sunshine snacks_sunshine cashew nuts light salt_unknown</t>
+          <t>shoon_shoon fatt cream crackers_unknown</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Sunshine Snacks</t>
+          <t>Shoon</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Sunshine Cashew Nuts Light Salt</t>
+          <t>SHOON FATT CREAM CRACKERS</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1.778846153846154</v>
+        <v>1.826923076923077</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Sunshine Snacks</t>
+          <t>Shoon</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Sunshine Cashew Nuts Light Salt</t>
+          <t>Shoon Fatt Cream Crackers</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>1.105769230769231</v>
+        <v>10.86538461538462</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="K48" t="n">
-        <v>60.86956521739126</v>
+        <v>-83.18584070796462</v>
       </c>
     </row>
     <row r="49">
@@ -2899,28 +2899,28 @@
         </is>
       </c>
       <c r="F49" t="n">
+        <v>1.778846153846154</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Sunshine Snacks</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Sunshine Cashew Nuts Light Salt</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>1.105769230769231</v>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Sunshine Snacks</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Sunshine Cashew Nuts Light Salt</t>
-        </is>
-      </c>
-      <c r="I49" t="n">
-        <v>1.778846153846154</v>
-      </c>
       <c r="J49" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
       <c r="K49" t="n">
-        <v>-37.83783783783782</v>
+        <v>60.86956521739126</v>
       </c>
     </row>
     <row r="50">
@@ -2936,34 +2936,34 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>triskits_triskits vanilla crackers_unknown</t>
+          <t>sunshine snacks_sunshine cashew nuts light salt_unknown</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Sunshine Snacks</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Sunshine Cashew Nuts Light Salt</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1.610576923076923</v>
+        <v>1.105769230769231</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Sunshine Snacks</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
+          <t>Sunshine Cashew Nuts Light Salt</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>1.346153846153846</v>
+        <v>1.778846153846154</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="K50" t="n">
-        <v>19.64285714285712</v>
+        <v>-37.83783783783782</v>
       </c>
     </row>
     <row r="51">
@@ -3014,7 +3014,7 @@
         </is>
       </c>
       <c r="I51" t="n">
-        <v>0.5769230769230769</v>
+        <v>1.346153846153846</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="K51" t="n">
-        <v>179.1666666666667</v>
+        <v>19.64285714285712</v>
       </c>
     </row>
     <row r="52">
@@ -3052,7 +3052,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1.346153846153846</v>
+        <v>1.610576923076923</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -3065,7 +3065,7 @@
         </is>
       </c>
       <c r="I52" t="n">
-        <v>1.610576923076923</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>-16.41791044776118</v>
+        <v>179.1666666666667</v>
       </c>
     </row>
     <row r="53">
@@ -3116,7 +3116,7 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>0.5769230769230769</v>
+        <v>1.610576923076923</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3124,7 +3124,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>133.3333333333334</v>
+        <v>-16.41791044776118</v>
       </c>
     </row>
     <row r="54">
@@ -3154,28 +3154,28 @@
         </is>
       </c>
       <c r="F54" t="n">
+        <v>1.346153846153846</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Triskits</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TRISKITS VANILLA CRACKERS</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
         <v>0.5769230769230769</v>
       </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Triskits</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>TRISKITS VANILLA CRACKERS</t>
-        </is>
-      </c>
-      <c r="I54" t="n">
-        <v>1.610576923076923</v>
-      </c>
       <c r="J54" t="inlineStr">
         <is>
           <t>both</t>
         </is>
       </c>
       <c r="K54" t="n">
-        <v>-64.17910447761194</v>
+        <v>133.3333333333334</v>
       </c>
     </row>
     <row r="55">
@@ -3218,7 +3218,7 @@
         </is>
       </c>
       <c r="I55" t="n">
-        <v>1.346153846153846</v>
+        <v>1.610576923076923</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -3226,7 +3226,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>-57.14285714285716</v>
+        <v>-64.17910447761194</v>
       </c>
     </row>
     <row r="56">
@@ -3242,34 +3242,34 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>wibisco_wibisco tea time chocolate_unknown</t>
+          <t>triskits_triskits vanilla crackers_unknown</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Wibisco</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Wibisco Tea Time Chocolate</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>4.086538461538462</v>
+        <v>0.5769230769230769</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Wibisco</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Wibisco Tea Time Chocolate</t>
+          <t>TRISKITS VANILLA CRACKERS</t>
         </is>
       </c>
       <c r="I56" t="n">
-        <v>0.4326923076923077</v>
+        <v>1.346153846153846</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
@@ -3277,7 +3277,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>844.4444444444445</v>
+        <v>-57.14285714285716</v>
       </c>
     </row>
     <row r="57">
@@ -3307,27 +3307,78 @@
         </is>
       </c>
       <c r="F57" t="n">
+        <v>4.086538461538462</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Wibisco</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Wibisco Tea Time Chocolate</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
         <v>0.4326923076923077</v>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>844.4444444444445</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Massy Stores Guyana</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>wibisco_wibisco tea time chocolate_unknown</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
         <is>
           <t>Wibisco</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Wibisco Tea Time Chocolate</t>
         </is>
       </c>
-      <c r="I57" t="n">
+      <c r="F58" t="n">
+        <v>0.4326923076923077</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Wibisco</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Wibisco Tea Time Chocolate</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
         <v>4.086538461538462</v>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>both</t>
-        </is>
-      </c>
-      <c r="K57" t="n">
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
         <v>-89.41176470588236</v>
       </c>
     </row>
@@ -3342,7 +3393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3405,31 +3456,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>bisco_bisco pan galleta clas integral_0.22</t>
+          <t>becky s_becky s tomato bread 190_0.19</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Bisco</t>
+          <t>Becky's</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bisco Pan Galleta Clas Integral</t>
+          <t>BECKY'S TOMATO BREAD | 190 g</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1.25</v>
+        <v>3.681564245810056</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -3444,31 +3495,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bisco_bisco pan galleta constanza_0.28</t>
+          <t>dove_dove vanilla ice cream bars coated with dark chocolate individually wrapped dessert 3 bars 16_0.45</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bisco</t>
+          <t>Dove</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bisco Pan Galleta Constanza</t>
+          <t>DOVE Vanilla Ice Cream Bars Coated With Dark Chocolate, Individually Wrapped Dessert, 3 Pack, Bars | 16 oz</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1.73</v>
+        <v>2.223463687150838</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -3483,31 +3534,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bisco_bisco pan pan integral mielpasas_0.38</t>
+          <t>dove_dove vanilla ice cream bars coated with milk chocolate individually wrapped dessert 3 bars 11_0.31</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Bisco</t>
+          <t>Dove</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bisco Pan Pan Integral Mielpasas</t>
+          <t>DOVE Vanilla Ice Cream Bars Coated With Milk Chocolate, Individually Wrapped Dessert, 3 Pack, Bars | 11 oz</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1.89</v>
+        <v>5.301675977653631</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -3522,31 +3573,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>bisco_bisco pan viga integral_0.45</t>
+          <t>kinder_kinder bueno milk chocolate and hazelnut cream 2 individually wrapped chocolate bars 11_0.31</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bisco</t>
+          <t>Kinder</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bisco Pan Viga Integral</t>
+          <t>Kinder Bueno Milk Chocolate and Hazelnut Cream, 2 Individually Wrapped Chocolate Bars, | 11 oz</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.3</v>
+        <v>2.955307262569832</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -3561,31 +3612,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>carrefour_bizcocho de chocolate conejo carrefour_unknown</t>
+          <t>kinder_liga kinder biscuits 12 36 maanden 300_0.3</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Kinder</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bizcocho De Chocolate Conejo Carrefour</t>
+          <t>LIGA KINDER BISCUITS 12-36 MAANDEN | 300 g</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.06</v>
+        <v>2.731843575418994</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -3600,31 +3651,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>carrefour_bizcocho frambuesa carrefour_0.15</t>
+          <t>kraft_kraft america s classic individually wrapped candy caramels bag 240_0.24</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Kraft</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bizcocho Frambuesa Carrefour</t>
+          <t>Kraft America's Classic Individually Wrapped Candy Caramels, Bag | 240 g</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.74</v>
+        <v>2.223463687150838</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
@@ -3639,31 +3690,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>carrefour_bizcocho ptit dej carrefour_0.4</t>
+          <t>nutella_nutella b ready 142_0.14</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nutella</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bizcocho Ptit Dej Carrefour</t>
+          <t>NUTELLA B-READY | 142 g</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3.96</v>
+        <v>1.223463687150838</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -3678,31 +3729,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>carrefour_bizcochos 6 carrefour classic de cereales_0.3</t>
+          <t>nutella_nutella biscuits 260_0.26</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nutella</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bizcochos 6 Carrefour Classic De Cereales</t>
+          <t>NUTELLA BISCUITS | 260 g</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.69</v>
+        <v>4.072625698324022</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
@@ -3717,31 +3768,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>carrefour_bizcochos carrefour classic naturales_0.3</t>
+          <t>santitas_santitas tortilla chips tortilla triangles 10_0.28</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Santitas</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bizcochos Carrefour Classic Naturales</t>
+          <t>SANTITAS TORTILLA CHIPS, TORTILLA TRIANGLES | 10 oz</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1.73</v>
+        <v>6.698324022346369</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -3756,31 +3807,31 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>carrefour_bizcochos carrefour naranja_0.15</t>
+          <t>toblerone_toblerone cheesecake 2x 225_0.17</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Toblerone</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bizcochos Carrefour Naranja</t>
+          <t>TOBLERONE CHEESECAKE 2X | 225 g</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.06</v>
+        <v>2.452513966480447</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -3795,31 +3846,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>carrefour_brownies carrefour pepites choco_0.28</t>
+          <t>twix_twix caramel cookie milk chocolate candy bars full size 3 02_0.09</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Twix</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Brownies Carrefour Pepites Choco</t>
+          <t>TWIX Caramel Cookie Milk Chocolate Candy Bars, Full Size, Pack | 3.02 oz</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.49</v>
+        <v>2.899441340782123</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -3834,31 +3885,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>carrefour_galleta carrefour chocograni chocolat noir_0.2</t>
+          <t>twix_twix milk chocolate caramel cookie candy bar share size 5 3_0.15</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Twix</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Chocograni Chocolat Noir</t>
+          <t>TWIX Milk Chocolate Caramel Cookie Candy Bar, Share Size, | 5.3 oz</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.61</v>
+        <v>2.508379888268156</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -3878,26 +3929,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>carrefour_galleta carrefour chocolate avellas_0.24</t>
+          <t>nutella_galletas b ready nutella_unknown</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nutella</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Chocolate Avellas</t>
+          <t>Galletas B Ready Nutella</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3.8</v>
+        <v>7.68</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -3917,26 +3968,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>carrefour_galleta carrefour chocolate caramelo_0.12</t>
+          <t>nutella_galletas biscuit nutella_0.34</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nutella</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Chocolate Caramelo</t>
+          <t>Galletas Biscuit Nutella</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3.01</v>
+        <v>7.53</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -3956,26 +4007,26 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Sirena</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>carrefour_galleta carrefour chocolate con leche_0.15</t>
+          <t>nutella_galletas b ready nutella_unknown</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nutella</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Chocolate Con Leche</t>
+          <t>Galletas B Ready Nutella</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.06</v>
+        <v>7.68</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -3990,31 +4041,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Guyana</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Massy Stores Guyana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>carrefour_galleta carrefour cocoa sin_0.12</t>
+          <t>chiefeez_chiefeez cheese ball_unknown</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Chiefeez</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Cocoa Sin Gluten</t>
+          <t>Chiefeez Cheese Ball</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3.64</v>
+        <v>0.4086538461538461</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -4029,31 +4080,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Guyana</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Massy Stores Guyana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>carrefour_galleta carrefour de pepitas de limon verde_0.1</t>
+          <t>shoon_shoon fatt veggie crackers_unknown</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Shoon</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Galleta Carrefour De Pepitas De Limon Verde</t>
+          <t>Shoon Fatt Veggie Crackers</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.85</v>
+        <v>3.557692307692307</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -4064,864 +4115,6 @@
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>carrefour_galleta carrefour dorada de guijarros de coco_0.12</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Dorada De Guijarros De Coco</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>carrefour_galleta carrefour mantequilla_0.12</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Mantequilla</t>
-        </is>
-      </c>
-      <c r="F20" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>carrefour_galleta carrefour praline de avellanas_0.11</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Praline De Avellanas</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>carrefour_galleta carrefour proteinas_0.15</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Proteinas</t>
-        </is>
-      </c>
-      <c r="F22" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>carrefour_galleta carrefour speculoos x2_0.17</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Speculoos X2</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>carrefour_galleta maiz con chocolate x carrefour bio_0.09</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Galleta Maiz Con Chocolate X Carrefour Bio</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>carrefour_galletas carrefour finas de gofre pura mantequilla_0.3</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Galletas Carrefour Finas De Gofre Pura Mantequilla</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>carrefour_galletas carrefour sensation tortillas simples_0.15</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Galletas Carrefour Sensation Tortillas Simples</t>
-        </is>
-      </c>
-      <c r="F26" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>carrefour_galletas de aperitivo carrefour classic galletas de emmental_0.1</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Galletas De Aperitivo Carrefour Classic Galletas De Emmental</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>carrefour_levadura para panes y brioches carrefour original_0.03</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Levadura Para Panes Y Brioches Carrefour Original</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>carrefour_surtido de galletas carrefour extra_0.2</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Surtido De Galletas Carrefour Extra</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>carrefour_tortillas de trigo carrefour sensation_0.37</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Tortillas De Trigo Carrefour Sensation</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Garrido</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>can can_galleta can can rell duplex_0.48</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Can Can</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Galleta Can Can Rell Duplex</t>
-        </is>
-      </c>
-      <c r="F31" t="n">
-        <v>1.82</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Jumbo</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>bisco_galletas biscuit mood rellenas de chocolate biscolata_0.12</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Bisco</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Galletas Biscuit Mood Rellenas De Chocolate Biscolata</t>
-        </is>
-      </c>
-      <c r="F32" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Merca Jumbo</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>bisco_galletas biscuit mood rellenas de chocolate biscolata_0.12</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Bisco</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Galletas Biscuit Mood Rellenas De Chocolate Biscolata</t>
-        </is>
-      </c>
-      <c r="F33" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Plaza Lama</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>bisco_bisco pan galleta clas integral_0.22</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Bisco</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Bisco Pan Galleta Clas Integral</t>
-        </is>
-      </c>
-      <c r="F34" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Plaza Lama</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>bisco_bisco pan galleta constanza_0.28</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Bisco</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Bisco Pan Galleta Constanza</t>
-        </is>
-      </c>
-      <c r="F35" t="n">
-        <v>1.82</v>
-      </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Plaza Lama</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>milka_choco wafer galletas de barquillo cubiertas de chocolate milka_0.18</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Milka</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Choco Wafer Galletas De Barquillo Cubiertas De Chocolate Milka</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>4.74</v>
-      </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Sirena</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>can can_galleta can can rell duplex_0.48</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Can Can</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Galleta Can Can Rell Duplex</t>
-        </is>
-      </c>
-      <c r="F37" t="n">
-        <v>1.93</v>
-      </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Sirena</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>milka_choco wafer galletas de barquillo cubiertas de chocolate milka_0.18</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Milka</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Choco Wafer Galletas De Barquillo Cubiertas De Chocolate Milka</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>5.07</v>
-      </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Sirena</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>milka_chocolate milka nutty wafer_0.27</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Milka</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Chocolate Milka Nutty Wafer</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Sirena</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>milka_galleta milka choco brownie_0.15</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Milka</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Galleta Milka Choco Brownie</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>5.23</v>
-      </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>left_only</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4934,7 +4127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4997,17 +4190,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>unknown_bisco pan galleta clas integral_0.22</t>
+          <t>liga_liga kinder biscuits 12 36 maanden 300_0.3</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -5015,16 +4208,16 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Liga</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Bisco Pan Galleta Clas Integral</t>
+          <t>LIGA KINDER BISCUITS 12-36 MAANDEN | 300 g</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>1.25</v>
+        <v>2.731843575418994</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -5036,17 +4229,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>unknown_bisco pan galleta constanza_0.28</t>
+          <t>unknown_becky s tomato bread 190_0.19</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -5059,11 +4252,11 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Bisco Pan Galleta Constanza</t>
+          <t>BECKY'S TOMATO BREAD | 190 g</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1.73</v>
+        <v>3.681564245810056</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -5075,17 +4268,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>unknown_bisco pan pan integral mielpasas_0.38</t>
+          <t>unknown_dove vanilla ice cream bars coated with dark chocolate individually wrapped dessert 3 bars 16_0.45</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -5098,11 +4291,11 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Bisco Pan Pan Integral Mielpasas</t>
+          <t>DOVE Vanilla Ice Cream Bars Coated With Dark Chocolate, Individually Wrapped Dessert, 3 Pack, Bars | 16 oz</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1.89</v>
+        <v>2.223463687150838</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -5114,17 +4307,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bravo</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>unknown_bisco pan viga integral_0.45</t>
+          <t>unknown_dove vanilla ice cream bars coated with milk chocolate individually wrapped dessert 3 bars 11_0.31</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -5137,11 +4330,11 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Bisco Pan Viga Integral</t>
+          <t>DOVE Vanilla Ice Cream Bars Coated With Milk Chocolate, Individually Wrapped Dessert, 3 Pack, Bars | 11 oz</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>2.3</v>
+        <v>5.301675977653631</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -5153,17 +4346,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>lu_galleta carrefour cocoa sin_0.12</t>
+          <t>unknown_kinder bueno milk chocolate and hazelnut cream 2 individually wrapped chocolate bars 11_0.31</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -5171,16 +4364,16 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Cocoa Sin Gluten</t>
+          <t>Kinder Bueno Milk Chocolate and Hazelnut Cream, 2 Individually Wrapped Chocolate Bars, | 11 oz</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>3.64</v>
+        <v>2.955307262569832</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -5192,17 +4385,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de chocolate conejo carrefour_unknown</t>
+          <t>unknown_kraft america s classic individually wrapped candy caramels bag 240_0.24</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -5215,11 +4408,11 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Bizcocho De Chocolate Conejo Carrefour</t>
+          <t>Kraft America's Classic Individually Wrapped Candy Caramels, Bag | 240 g</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>2.06</v>
+        <v>2.223463687150838</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -5231,17 +4424,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>unknown_bizcocho frambuesa carrefour_0.15</t>
+          <t>unknown_nutella b ready 142_0.14</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -5254,11 +4447,11 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Bizcocho Frambuesa Carrefour</t>
+          <t>NUTELLA B-READY | 142 g</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1.74</v>
+        <v>1.223463687150838</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -5270,17 +4463,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>unknown_bizcocho ptit dej carrefour_0.4</t>
+          <t>unknown_nutella biscuits 260_0.26</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -5293,11 +4486,11 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Bizcocho Ptit Dej Carrefour</t>
+          <t>NUTELLA BISCUITS | 260 g</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>3.96</v>
+        <v>4.072625698324022</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -5309,17 +4502,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>unknown_bizcochos 6 carrefour classic de cereales_0.3</t>
+          <t>unknown_santitas tortilla chips tortilla triangles 10_0.28</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -5332,11 +4525,11 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Bizcochos 6 Carrefour Classic De Cereales</t>
+          <t>SANTITAS TORTILLA CHIPS, TORTILLA TRIANGLES | 10 oz</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2.69</v>
+        <v>6.698324022346369</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -5348,17 +4541,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>unknown_bizcochos carrefour classic naturales_0.3</t>
+          <t>unknown_toblerone cheesecake 2x 225_0.17</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -5371,11 +4564,11 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Bizcochos Carrefour Classic Naturales</t>
+          <t>TOBLERONE CHEESECAKE 2X | 225 g</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1.73</v>
+        <v>2.452513966480447</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -5387,17 +4580,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>unknown_bizcochos carrefour naranja_0.15</t>
+          <t>unknown_twix caramel cookie milk chocolate candy bars full size 3 02_0.09</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -5410,11 +4603,11 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Bizcochos Carrefour Naranja</t>
+          <t>TWIX Caramel Cookie Milk Chocolate Candy Bars, Full Size, Pack | 3.02 oz</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>2.06</v>
+        <v>2.899441340782123</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -5426,17 +4619,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Super Food Aruba</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>unknown_brownies carrefour pepites choco_0.28</t>
+          <t>unknown_twix milk chocolate caramel cookie candy bar share size 5 3_0.15</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -5449,11 +4642,11 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Brownies Carrefour Pepites Choco</t>
+          <t>TWIX Milk Chocolate Caramel Cookie Candy Bar, Share Size, | 5.3 oz</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>3.49</v>
+        <v>2.508379888268156</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -5470,12 +4663,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>unknown_galleta carrefour chocograni chocolat noir_0.2</t>
+          <t>unknown_galletas b ready nutella_unknown</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -5488,11 +4681,11 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Chocograni Chocolat Noir</t>
+          <t>Galletas B Ready Nutella</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2.61</v>
+        <v>7.68</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -5509,12 +4702,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>unknown_galleta carrefour chocolate avellas_0.24</t>
+          <t>unknown_galletas biscuit nutella_0.34</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -5527,11 +4720,11 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Chocolate Avellas</t>
+          <t>Galletas Biscuit Nutella</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>3.8</v>
+        <v>7.53</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -5548,12 +4741,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Sirena</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>unknown_galleta carrefour chocolate caramelo_0.12</t>
+          <t>unknown_galletas b ready nutella_unknown</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -5566,11 +4759,11 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Chocolate Caramelo</t>
+          <t>Galletas B Ready Nutella</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>3.01</v>
+        <v>7.68</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -5582,17 +4775,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Guyana</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Massy Stores Guyana</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>unknown_galleta carrefour chocolate con leche_0.15</t>
+          <t>unknown_chiefeez cheese ball_unknown</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -5605,11 +4798,11 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Chocolate Con Leche</t>
+          <t>Chiefeez Cheese Ball</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>2.06</v>
+        <v>0.4086538461538461</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -5621,17 +4814,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Guyana</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Massy Stores Guyana</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>unknown_galleta carrefour de pepitas de limon verde_0.1</t>
+          <t>unknown_shoon fatt butter crackers_unknown</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -5644,11 +4837,11 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Galleta Carrefour De Pepitas De Limon Verde</t>
+          <t>SHOON FATT BUTTER CRACKERS</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>2.85</v>
+        <v>1.778846153846154</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -5660,17 +4853,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Guyana</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Massy Stores Guyana</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>unknown_galleta carrefour dorada de guijarros de coco_0.12</t>
+          <t>unknown_shoon fatt veggie crackers_unknown</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -5683,11 +4876,11 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Galleta Carrefour Dorada De Guijarros De Coco</t>
+          <t>Shoon Fatt Veggie Crackers</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>0.79</v>
+        <v>3.557692307692307</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -5695,825 +4888,6 @@
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>unknown_galleta carrefour mantequilla_0.12</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Mantequilla</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>unknown_galleta carrefour praline de avellanas_0.11</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Praline De Avellanas</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>unknown_galleta carrefour proteinas_0.15</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Proteinas</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>3.09</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>unknown_galleta carrefour speculoos x2_0.17</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Galleta Carrefour Speculoos X2</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>unknown_galleta maiz con chocolate x carrefour bio_0.09</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Galleta Maiz Con Chocolate X Carrefour Bio</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>unknown_galletas carrefour finas de gofre pura mantequilla_0.3</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Galletas Carrefour Finas De Gofre Pura Mantequilla</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>unknown_galletas carrefour sensation tortillas simples_0.15</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Galletas Carrefour Sensation Tortillas Simples</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>unknown_galletas de aperitivo carrefour classic galletas de emmental_0.1</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Galletas De Aperitivo Carrefour Classic Galletas De Emmental</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>unknown_levadura para panes y brioches carrefour original_0.03</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Levadura Para Panes Y Brioches Carrefour Original</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>unknown_surtido de galletas carrefour extra_0.2</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Surtido De Galletas Carrefour Extra</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Carrefour</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>unknown_tortillas de trigo carrefour sensation_0.37</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Tortillas De Trigo Carrefour Sensation</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Garrido</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>unknown_galleta can can rell duplex_0.48</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Galleta Can Can Rell Duplex</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>1.82</v>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Jumbo</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>unknown_galletas biscuit mood rellenas de chocolate biscolata_0.12</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Galletas Biscuit Mood Rellenas De Chocolate Biscolata</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Merca Jumbo</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>unknown_galletas biscuit mood rellenas de chocolate biscolata_0.12</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Galletas Biscuit Mood Rellenas De Chocolate Biscolata</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Plaza Lama</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>unknown_bisco pan galleta clas integral_0.22</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Bisco Pan Galleta Clas Integral</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Plaza Lama</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>unknown_bisco pan galleta constanza_0.28</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Bisco Pan Galleta Constanza</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>1.82</v>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Plaza Lama</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>unknown_choco wafer galletas de barquillo cubiertas de chocolate milka_0.18</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Choco Wafer Galletas De Barquillo Cubiertas De Chocolate Milka</t>
-        </is>
-      </c>
-      <c r="I36" t="n">
-        <v>4.74</v>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Sirena</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>unknown_choco wafer galletas de barquillo cubiertas de chocolate milka_0.18</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Choco Wafer Galletas De Barquillo Cubiertas De Chocolate Milka</t>
-        </is>
-      </c>
-      <c r="I37" t="n">
-        <v>5.07</v>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Sirena</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>unknown_chocolate milka nutty wafer_0.27</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Chocolate Milka Nutty Wafer</t>
-        </is>
-      </c>
-      <c r="I38" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Sirena</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>unknown_galleta can can rell duplex_0.48</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Galleta Can Can Rell Duplex</t>
-        </is>
-      </c>
-      <c r="I39" t="n">
-        <v>1.93</v>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Dominican Republic</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Sirena</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>unknown_galleta milka choco brownie_0.15</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Galleta Milka Choco Brownie</t>
-        </is>
-      </c>
-      <c r="I40" t="n">
-        <v>5.23</v>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>right_only</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily Caribbean retail update 2026-06-07
</commit_message>
<xml_diff>
--- a/streamlit_data/price_alerts.xlsx
+++ b/streamlit_data/price_alerts.xlsx
@@ -3546,7 +3546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3614,26 +3614,26 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Bravo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ecovida_galleta ecovida sin coco_0.15</t>
+          <t>bon_helados bon bizcocho_0.26</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ecovida</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Galleta Ecovida Sin Gluten Coco</t>
+          <t>Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.41</v>
+        <v>3.95</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -3653,26 +3653,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Bravo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ecovida_galleta sin berrie ecovida_0.15</t>
+          <t>dante_galletas cubanas dante con ajo_0.27</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ecovida</t>
+          <t>Dante</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Galleta Sin Gluten Berrie Ecovida</t>
+          <t>Galletas Cubanas Dante Con Ajo</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>3.41</v>
+        <v>1.89</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -3692,26 +3692,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Bravo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ecovida_galletas sin azucar rellenas de higo ecovida_0.15</t>
+          <t>dante_galletas cubanas dante_0.27</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ecovida</t>
+          <t>Dante</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Galletas Sin Azucar Rellenas De Higo Ecovida</t>
+          <t>Galletas Cubanas Dante</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2.22</v>
+        <v>1.89</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -3731,26 +3731,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Bravo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>gri gri_galleta integral con ajonjoli gri gri_unknown</t>
+          <t>mamut_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Gri Gri</t>
+          <t>Mamut</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Galleta Integral Con Ajonjoli Gri Gri</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1.82</v>
+        <v>0.48</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
@@ -3770,26 +3770,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>mestemacher_pan integral de centeno con semillas de calabaza mestemacher_0.5</t>
+          <t>bon_helado helados bon bizcocho_0.52</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Mestemacher</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Pan Integral De Centeno Con Semillas De Calabaza Mestemacher</t>
+          <t>Helado Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.85</v>
+        <v>5.78</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -3809,26 +3809,26 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>mestemacher_pan integral de centeno con semillas de girasol mestemacher_0.5</t>
+          <t>bon_helados bon bizcocho_0.26</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mestemacher</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pan Integral De Centeno Con Semillas De Girasol Mestemacher</t>
+          <t>Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.85</v>
+        <v>3.71</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
@@ -3848,26 +3848,26 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>over the top_capacillos desechables para hornear cupcakes colores mixtos over the top_unknown</t>
+          <t>bon_paleta bon de bizcocho_unknown</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Over The Top</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Capacillos Desechables Para Hornear Cupcakes Colores Mixtos Over The Top</t>
+          <t>Paleta Bon De Bizcocho</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>4.44</v>
+        <v>0.63</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -3887,26 +3887,26 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>over the top_capacillos grandes desechables para hornear cupcakes over the top_unknown</t>
+          <t>gavotte_galleta gavotte dentelle_0.12</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Over The Top</t>
+          <t>Gavotte</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Capacillos Grandes Desechables Para Hornear Cupcakes Over The Top</t>
+          <t>Galleta Gavotte Dentelle</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.22</v>
+        <v>3.64</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
@@ -3926,22 +3926,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>over the top_capacillos para mini cupcakes over the top_unknown</t>
+          <t>mocano_galleta manteca mocano_unknown</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Over The Top</t>
+          <t>Mocano</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Capacillos Para Mini Cupcakes Over The Top</t>
+          <t>Galleta Manteca Mocano</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -3965,26 +3965,26 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>spongy_bizcocho de vainilla spongy_0.15</t>
+          <t>pozuelo_galleta pozuelo chiky chocolate_unknown</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Spongy</t>
+          <t>Pozuelo</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Galleta Pozuelo Chiky Chocolate</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1.35</v>
+        <v>3.58</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -4004,26 +4004,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>sweet ps_bizcocho de guineo rebanado sweet ps_0.45</t>
+          <t>pozuelo_galleta pozuelo cremas chocolate_unknown</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Pozuelo</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Bizcocho De Guineo Rebanado Sweet Ps</t>
+          <t>Galleta Pozuelo Cremas Chocolate</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>6.02</v>
+        <v>1.88</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -4043,26 +4043,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sweet ps_bizcocho marmol rabanado sweet ps_0.45</t>
+          <t>pozuelo_galleta pozuelo cremas fresa_unknown</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Pozuelo</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bizcocho Marmol Rabanado Sweet Ps</t>
+          <t>Galleta Pozuelo Cremas Fresa</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>6.02</v>
+        <v>1.88</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
@@ -4082,26 +4082,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>sweet ps_bizcocho pudin de mantequilla y canela rebanao sweet ps_0.45</t>
+          <t>pozuelo_galleta pozuelo vainilla chocolate_0.3</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Pozuelo</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bizcocho Pudin De Mantequilla Y Canela Rebanao Sweet Ps</t>
+          <t>Galleta Pozuelo Vainilla Chocolate</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>6.02</v>
+        <v>1.82</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
@@ -4121,26 +4121,26 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>bgourmet_pan brioche chocolatechip bgourmet_0.4</t>
+          <t>renata_galleta maizena renata_0.36</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BGourmet</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Pan Brioche Chocolatechip Bgourmet</t>
+          <t>Galleta Maizena Renata</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>5.85</v>
+        <v>2.06</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -4160,26 +4160,26 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>bgourmet_pan brioche lonjeado bgourmet_0.5</t>
+          <t>renata_galleta renata wafer choc_0.12</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>BGourmet</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Pan Brioche Lonjeado Bgourmet</t>
+          <t>Galleta Renata Wafer Choc</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>6.85</v>
+        <v>0.95</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -4199,26 +4199,26 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>dbl_galleta de chocolate chip vegana dbl_0.07</t>
+          <t>renata_mezcla para bizcocho renata coco_0.4</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>DBL</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Vegana Dbl</t>
+          <t>Mezcla Para Bizcocho Renata Coco</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3.39</v>
+        <v>2.14</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -4238,26 +4238,26 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>dbl_galleta de chocolate chip vegana dbl_0.34</t>
+          <t>renata_mezcla para bizcocho renata limon_0.4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DBL</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Vegana Dbl</t>
+          <t>Mezcla Para Bizcocho Renata Limon</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>6.4</v>
+        <v>2.14</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -4277,26 +4277,26 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>green is my thing_galleta de chocolate chip artesanal green is my thing_unknown</t>
+          <t>renata_mezcla para bizcocho renata maiz_0.4</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Green Is My Thing</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Artesanal Green Is My Thing</t>
+          <t>Mezcla Para Bizcocho Renata Maiz</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>3.55</v>
+        <v>2.14</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -4316,26 +4316,26 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>green is my thing_galletas artesanales de avena green is my thing_unknown</t>
+          <t>renata_mezcla para bizcocho renata naranja_0.4</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Green Is My Thing</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Galletas Artesanales De Avena Green Is My Thing</t>
+          <t>Mezcla Para Bizcocho Renata Naranja</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3.55</v>
+        <v>2.14</v>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -4355,26 +4355,26 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>gri gri_galleta integral con ajonjoli gri gri_unknown</t>
+          <t>renata_mezcla para bizcocho renata pina_0.4</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Gri Gri</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Galleta Integral Con Ajonjoli Gri Gri</t>
+          <t>Mezcla Para Bizcocho Renata Pina</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1.81</v>
+        <v>2.14</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -4394,26 +4394,26 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ita abu_galletas artesanales de vainilla y guayaba ita abu_unknown</t>
+          <t>renata_mezcla para bizcocho renata vainilla_0.4</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Ita Abu</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Galletas Artesanales De Vainilla Y Guayaba Ita Abu</t>
+          <t>Mezcla Para Bizcocho Renata Vainilla</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.44</v>
+        <v>2.14</v>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
@@ -4433,26 +4433,26 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>mandul_mini muffins choco chips mandul_0.2</t>
+          <t>choco wow_galletas sandwich chocolate choco wow 10 und_0.48</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mandul</t>
+          <t>Choco Wow</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mini Muffins Choco Chips Mandul</t>
+          <t>Galletas Sandwich Chocolate Choco Wow 10 Und</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>3.79</v>
+        <v>2.14</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
@@ -4472,26 +4472,26 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>mandul_mini muffins choco stars mandul_0.21</t>
+          <t>lago_galleta lago mini party cacao_0.12</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Mandul</t>
+          <t>Lago</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Mini Muffins Choco Stars Mandul</t>
+          <t>Galleta Lago Mini Party Cacao</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3.79</v>
+        <v>1.66</v>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
@@ -4511,26 +4511,26 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>mandul_mini muffins rellenos de fresa mandul_0.21</t>
+          <t>mamut_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Mandul</t>
+          <t>Mamut</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Mini Muffins Rellenos De Fresa Mandul</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.79</v>
+        <v>0.46</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
@@ -4550,26 +4550,26 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>repeat_galleta de avena vegan repeat_0.04</t>
+          <t>muuu_galletas de chocolate muuu con crema sabor a vainilla_unknown</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Repeat</t>
+          <t>Muuu</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Galleta De Avena Vegan Repeat</t>
+          <t>Galletas De Chocolate Muuu Con Crema Sabor A Vainilla</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2.12</v>
+        <v>2.69</v>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
@@ -4589,26 +4589,26 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>repeat_galleta de avena vegan repeat_0.1</t>
+          <t>supermoist_mezcla para bizcocho de zanahoria supermoist_0.43</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Repeat</t>
+          <t>SuperMoist</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Galleta De Avena Vegan Repeat</t>
+          <t>Mezcla Para Bizcocho De Zanahoria Supermoist</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>4.74</v>
+        <v>4.99</v>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
@@ -4628,26 +4628,26 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>spongy_bizcocho de vainilla spongy_0.15</t>
+          <t>vaquita rica_leche sabor bizcocho vaquita rica uht_unknown</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Spongy</t>
+          <t>Vaquita Rica</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Leche Sabor Bizcocho Vaquita Rica Uht</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1.17</v>
+        <v>0.48</v>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
@@ -4667,26 +4667,26 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Jumbo</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>sweet ps_cup cake de vainilla con chispas sweet ps_0.28</t>
+          <t>mamut_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Mamut</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Cup Cake De Vainilla Con Chispas Sweet Ps</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>5.05</v>
+        <v>0.47</v>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
@@ -4706,26 +4706,26 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Jumbo</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sweet ps_mini brownies sweet ps_0.3</t>
+          <t>quest_barra de proteina sabor brownie de chocolate quest_0.06</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Quest</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Mini Brownies Sweet Ps</t>
+          <t>Barra De Proteina Sabor Brownie De Chocolate Quest</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>5.69</v>
+        <v>4.72</v>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -4745,26 +4745,26 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>bgourmet_pan brioche chocolatechip bgourmet_0.4</t>
+          <t>bon_helado bizcocho bon 2 pintas_unknown</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>BGourmet</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Pan Brioche Chocolatechip Bgourmet</t>
+          <t>Helado Bizcocho Bon 2 Pintas</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>5.86</v>
+        <v>5.45</v>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
@@ -4784,26 +4784,26 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>bgourmet_pan brioche lonjeado bgourmet_0.5</t>
+          <t>bon_helados bon bizcocho_0.26</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>BGourmet</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Pan Brioche Lonjeado Bgourmet</t>
+          <t>Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>6.86</v>
+        <v>3.69</v>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
@@ -4823,26 +4823,26 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>dbl_galleta de chocolate chip vegana dbl_0.07</t>
+          <t>choco wow_galletas sandwich chocolate choco wow 10 und_0.48</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>DBL</t>
+          <t>Choco Wow</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Vegana Dbl</t>
+          <t>Galletas Sandwich Chocolate Choco Wow 10 Und</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.41</v>
+        <v>2.2</v>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
@@ -4862,26 +4862,26 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>dbl_galleta de chocolate chip vegana dbl_0.34</t>
+          <t>mamut_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>DBL</t>
+          <t>Mamut</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Vegana Dbl</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>6.42</v>
+        <v>0.46</v>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
@@ -4901,26 +4901,26 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ecovida_galleta de chocolate chips sin ecovida_0.15</t>
+          <t>popcorners_tortillas chips kettle corn popcorners_0.14</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Ecovida</t>
+          <t>PopCorners</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chips Sin Gluten Ecovida</t>
+          <t>Tortillas Chips Kettle Corn Popcorners</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.72</v>
+        <v>3.63</v>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
@@ -4940,26 +4940,26 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ecovida_galletas sin azucar rellenas de higo ecovida_0.15</t>
+          <t>quest_barra de proteina sabor brownie de chocolate quest_0.06</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Ecovida</t>
+          <t>Quest</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Galletas Sin Azucar Rellenas De Higo Ecovida</t>
+          <t>Barra De Proteina Sabor Brownie De Chocolate Quest</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.65</v>
+        <v>4.71</v>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
@@ -4984,21 +4984,21 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>green is my thing_galleta de chocolate chip artesanal green is my thing_unknown</t>
+          <t>axa_galletas cookie n cream axa_0.14</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Green Is My Thing</t>
+          <t>AXA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Artesanal Green Is My Thing</t>
+          <t>Galletas Cookie N Cream Axa</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.56</v>
+        <v>4.69</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
@@ -5023,21 +5023,21 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>green is my thing_galletas artesanales de avena green is my thing_unknown</t>
+          <t>lotus_galleta de mantequilla lotus_0.25</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Green Is My Thing</t>
+          <t>Lotus</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Galletas Artesanales De Avena Green Is My Thing</t>
+          <t>Galleta De Mantequilla Lotus</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>3.56</v>
+        <v>4.28</v>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
@@ -5062,21 +5062,21 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ita abu_galletas artesanales de vainilla y guayaba ita abu_unknown</t>
+          <t>lotus_galleta de mantequilla rellena de chocolate lotus_0.15</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Ita Abu</t>
+          <t>Lotus</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Galletas Artesanales De Vainilla Y Guayaba Ita Abu</t>
+          <t>Galleta De Mantequilla Rellena De Chocolate Lotus</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2.46</v>
+        <v>3.49</v>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr"/>
@@ -5101,21 +5101,21 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>mandul_mini muffins choco chips mandul_0.2</t>
+          <t>mamut_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Mandul</t>
+          <t>Mamut</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Mini Muffins Choco Chips Mandul</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.8</v>
+        <v>0.47</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr"/>
@@ -5140,21 +5140,21 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>mandul_mini muffins choco stars mandul_0.21</t>
+          <t>new york style_bagel crisps plain new york style_0.2</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Mandul</t>
+          <t>New York Style</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Mini Muffins Choco Stars Mandul</t>
+          <t>Bagel Crisps Plain New York Style</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.8</v>
+        <v>3.56</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
@@ -5179,21 +5179,21 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>mandul_mini muffins rellenos de fresa mandul_0.21</t>
+          <t>new york style_bagel crisps sea salt new york style_0.2</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Mandul</t>
+          <t>New York Style</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Mini Muffins Rellenos De Fresa Mandul</t>
+          <t>Bagel Crisps Sea Salt New York Style</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.8</v>
+        <v>3.56</v>
       </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
@@ -5218,21 +5218,21 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>mestemacher_pan integral de centeno con semillas de calabaza mestemacher_0.5</t>
+          <t>popcorners_tortillas chips kettle corn popcorners_0.14</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Mestemacher</t>
+          <t>PopCorners</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Pan Integral De Centeno Con Semillas De Calabaza Mestemacher</t>
+          <t>Tortillas Chips Kettle Corn Popcorners</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>2.85</v>
+        <v>3.64</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
@@ -5257,21 +5257,21 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>mestemacher_pan integral de centeno con semillas de girasol mestemacher_0.5</t>
+          <t>quest_barra de proteina sabor brownie de chocolate quest_0.06</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Mestemacher</t>
+          <t>Quest</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Pan Integral De Centeno Con Semillas De Girasol Mestemacher</t>
+          <t>Barra De Proteina Sabor Brownie De Chocolate Quest</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.85</v>
+        <v>4.72</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr"/>
@@ -5296,21 +5296,21 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>over the top_capacillos desechables para hornear cupcakes colores mixtos over the top_unknown</t>
+          <t>supermoist_mezcla para bizcocho de zanahoria supermoist_0.43</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Over The Top</t>
+          <t>SuperMoist</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Capacillos Desechables Para Hornear Cupcakes Colores Mixtos Over The Top</t>
+          <t>Mezcla Para Bizcocho De Zanahoria Supermoist</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>4.44</v>
+        <v>4.83</v>
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
@@ -5335,21 +5335,21 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>over the top_capacillos grandes desechables para hornear cupcakes over the top_unknown</t>
+          <t>vaquita rica_leche sabor bizcocho vaquita rica uht_unknown</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Over The Top</t>
+          <t>Vaquita Rica</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Capacillos Grandes Desechables Para Hornear Cupcakes Over The Top</t>
+          <t>Leche Sabor Bizcocho Vaquita Rica Uht</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>2.22</v>
+        <v>0.46</v>
       </c>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
@@ -5369,26 +5369,26 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>repeat_galleta de avena vegan repeat_0.04</t>
+          <t>bon_helado bon de bizcocho_0.52</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Repeat</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Galleta De Avena Vegan Repeat</t>
+          <t>Helado Bon De Bizcocho</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>2.14</v>
+        <v>6.32</v>
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
@@ -5408,26 +5408,26 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>repeat_galleta de avena vegan repeat_0.1</t>
+          <t>bon_helados bon bizcocho_0.26</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Repeat</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Galleta De Avena Vegan Repeat</t>
+          <t>Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>4.75</v>
+        <v>4.26</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
@@ -5447,26 +5447,26 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>sheila s_galletas brownie brittle chocolate chips sheila gs_0.14</t>
+          <t>bon_paleta bon de bizcocho_unknown</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Sheila G's</t>
+          <t>Bon</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Chocolate Chips Sheila Gs</t>
+          <t>Paleta Bon De Bizcocho</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>4.75</v>
+        <v>0.71</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
@@ -5486,26 +5486,26 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>sheila s_galletas brownie brittle dark chocolate sea salt sheila gs_0.14</t>
+          <t>dante_galletas cubanas dante con ajo_0.27</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Sheila G's</t>
+          <t>Dante</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Dark Chocolate Sea Salt Sheila Gs</t>
+          <t>Galletas Cubanas Dante Con Ajo</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>4.75</v>
+        <v>2.14</v>
       </c>
       <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr"/>
@@ -5525,26 +5525,26 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>sheila s_galletas brownie brittle salted caramel sheila gs_0.14</t>
+          <t>dante_galletas cubanas dante_0.27</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Sheila G's</t>
+          <t>Dante</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Salted Caramel Sheila Gs</t>
+          <t>Galletas Cubanas Dante</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>4.75</v>
+        <v>2.14</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
@@ -5564,26 +5564,26 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>spongy_bizcocho de vainilla spongy_0.15</t>
+          <t>lago_galleta wafers lago poker con avellanas 5 und_0.22</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Spongy</t>
+          <t>Lago</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Galleta Wafers Lago Poker Con Avellanas 5 Und</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1.35</v>
+        <v>2.99</v>
       </c>
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr"/>
@@ -5603,26 +5603,26 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>sweet ps_bizcocho de guineo rebanado sweet ps_0.45</t>
+          <t>loacker_galleta wafers loacker sabor a coconut_0.04</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Loacker</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Bizcocho De Guineo Rebanado Sweet Ps</t>
+          <t>Galleta Wafers Loacker Sabor A Coconut</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>6.02</v>
+        <v>1.09</v>
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr"/>
@@ -5642,26 +5642,26 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>sweet ps_bizcocho de limon rebanado sweet ps_0.45</t>
+          <t>loacker_galleta wafers loacker sabor a cremkakao_0.04</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Loacker</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Bizcocho De Limon Rebanado Sweet Ps</t>
+          <t>Galleta Wafers Loacker Sabor A Cremkakao</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>6.02</v>
+        <v>1.09</v>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
@@ -5681,26 +5681,26 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>sweet ps_bizcocho marmol rabanado sweet ps_0.45</t>
+          <t>loacker_galleta wafers loacker sabor a napolitaner_0.04</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Loacker</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Bizcocho Marmol Rabanado Sweet Ps</t>
+          <t>Galleta Wafers Loacker Sabor A Napolitaner</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>6.02</v>
+        <v>1.09</v>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
@@ -5720,26 +5720,26 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>sweet ps_bizcocho pudin de mantequilla y canela rebanao sweet ps_0.45</t>
+          <t>loacker_galleta wafers loacker sabor a vainilla_0.04</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Loacker</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bizcocho Pudin De Mantequilla Y Canela Rebanao Sweet Ps</t>
+          <t>Galleta Wafers Loacker Sabor A Vainilla</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>6.02</v>
+        <v>1.09</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
@@ -5759,26 +5759,26 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sweet ps_cup cake de vainilla con chispas sweet ps_0.28</t>
+          <t>mamut_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Mamut</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Cup Cake De Vainilla Con Chispas Sweet Ps</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>5.07</v>
+        <v>0.48</v>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
@@ -5798,26 +5798,26 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>sweet ps_mini brownies sweet ps_0.3</t>
+          <t>muuu_galletas de chocolate muuu con crema sabor a vainilla_unknown</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>Muuu</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Mini Brownies Sweet Ps</t>
+          <t>Galletas De Chocolate Muuu Con Crema Sabor A Vainilla</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>5.7</v>
+        <v>2.76</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
@@ -5837,26 +5837,26 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>sweet ps_mini cup cakes red velvet sweet ps_unknown</t>
+          <t>popcorners_tortillas chips kettle corn popcorners_0.14</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Sweet Ps</t>
+          <t>PopCorners</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Mini Cup Cakes Red Velvet Sweet Ps</t>
+          <t>Tortillas Chips Kettle Corn Popcorners</t>
         </is>
       </c>
       <c r="F59" t="n">
-        <v>6.32</v>
+        <v>3.64</v>
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
@@ -5881,21 +5881,21 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>spongy_bizcocho de vainilla spongy_0.15</t>
+          <t>quest_barra de proteina sabor brownie de chocolate quest_0.06</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Spongy</t>
+          <t>Quest</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Barra De Proteina Sabor Brownie De Chocolate Quest</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>1.35</v>
+        <v>4.72</v>
       </c>
       <c r="G60" t="inlineStr"/>
       <c r="H60" t="inlineStr"/>
@@ -5915,26 +5915,26 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Plaza Lama</t>
+          <t>Sirena</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>spongy_bizcocho spongy vainilla_0.23</t>
+          <t>bridge_galletas bridge wafer naranja_0.3</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Spongy</t>
+          <t>Bridge</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Bizcocho Spongy Vainilla</t>
+          <t>Galletas Bridge Wafer Naranja</t>
         </is>
       </c>
       <c r="F61" t="n">
-        <v>1.35</v>
+        <v>1.51</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr"/>
@@ -5954,26 +5954,26 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ritmo</t>
+          <t>Sirena</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>spongy_bizcocho de vainilla spongy_0.15</t>
+          <t>cheez it_galleta snapd doble cheddar cheez it_0.21</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Spongy</t>
+          <t>Cheez-It</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Galleta Snapd Doble Cheddar Cheez It</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>1.09</v>
+        <v>4.6</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
@@ -5998,21 +5998,21 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ecovida_galleta ecovida sin coco_0.15</t>
+          <t>choco wow_galletas sandwich chocolate choco wow 10 und_0.48</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Ecovida</t>
+          <t>Choco Wow</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Galleta Ecovida Sin Gluten Coco</t>
+          <t>Galletas Sandwich Chocolate Choco Wow 10 Und</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>3.72</v>
+        <v>2.22</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
@@ -6037,21 +6037,21 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ecovida_galleta sin berrie ecovida_0.15</t>
+          <t>jules destrooper_galleta de mantequilla jules destrooper_0.1</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Ecovida</t>
+          <t>Jules Destrooper</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Galleta Sin Gluten Berrie Ecovida</t>
+          <t>Galleta De Mantequilla Jules Destrooper</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>3.72</v>
+        <v>3.96</v>
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
@@ -6076,21 +6076,21 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>sheila s_galletas brownie brittle chocolate chips sheila gs_0.14</t>
+          <t>lago_galleta lago mini party cacao_0.12</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Sheila G's</t>
+          <t>Lago</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Chocolate Chips Sheila Gs</t>
+          <t>Galleta Lago Mini Party Cacao</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>5.15</v>
+        <v>2.06</v>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr"/>
@@ -6115,21 +6115,21 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>sheila s_galletas brownie brittle dark chocolate sea salt sheila gs_0.14</t>
+          <t>lago_galleta wafers lago wafers mini party avellanas_0.12</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Sheila G's</t>
+          <t>Lago</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Dark Chocolate Sea Salt Sheila Gs</t>
+          <t>Galleta Wafers Lago Wafers Mini Party Avellanas</t>
         </is>
       </c>
       <c r="F66" t="n">
-        <v>5.15</v>
+        <v>2.06</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
@@ -6154,21 +6154,21 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>sheila s_galletas brownie brittle salted caramel sheila gs_0.14</t>
+          <t>lotus_galleta de mantequilla lotus_0.25</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Sheila G's</t>
+          <t>Lotus</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Salted Caramel Sheila Gs</t>
+          <t>Galleta De Mantequilla Lotus</t>
         </is>
       </c>
       <c r="F67" t="n">
-        <v>5.15</v>
+        <v>4.28</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
@@ -6179,6 +6179,123 @@
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Dominican Republic</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Sirena</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>mamut_galletas de chocolate y malvavisco mamut_0.03</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Mamut</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>left_only</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Dominican Republic</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Sirena</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>popcorners_tortillas chips kettle corn popcorners_0.14</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>PopCorners</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Tortillas Chips Kettle Corn Popcorners</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>left_only</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Massy Stores Guyana</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>cheez it_cheez it original 1 5oz_0.04</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Cheez-It</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Cheez-It Original  1.5oz</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1.201923076923077</v>
+      </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>left_only</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6191,7 +6308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6259,12 +6376,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Bravo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>lu_galleta ecovida sin coco_0.15</t>
+          <t>unknown_galletas cubanas dante con ajo_0.27</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -6272,16 +6389,16 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Galleta Ecovida Sin Gluten Coco</t>
+          <t>Galletas Cubanas Dante Con Ajo</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>3.41</v>
+        <v>1.89</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -6298,12 +6415,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Bravo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>lu_galleta sin berrie ecovida_0.15</t>
+          <t>unknown_galletas cubanas dante_0.27</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -6311,16 +6428,16 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Galleta Sin Gluten Berrie Ecovida</t>
+          <t>Galletas Cubanas Dante</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>3.41</v>
+        <v>1.89</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -6337,12 +6454,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Carrefour</t>
+          <t>Bravo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>unknown_galletas sin azucar rellenas de higo ecovida_0.15</t>
+          <t>unknown_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -6355,11 +6472,11 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Galletas Sin Azucar Rellenas De Higo Ecovida</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2.22</v>
+        <v>0.48</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -6376,12 +6493,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Bravo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de guineo rebanado sweet ps_0.45</t>
+          <t>unknown_helados bon bizcocho_0.26</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -6394,11 +6511,11 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Bizcocho De Guineo Rebanado Sweet Ps</t>
+          <t>Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>6.02</v>
+        <v>3.95</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -6415,12 +6532,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de vainilla spongy_0.15</t>
+          <t>unknown_galleta gavotte dentelle_0.12</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -6433,11 +6550,11 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Galleta Gavotte Dentelle</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1.35</v>
+        <v>3.64</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -6454,12 +6571,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>unknown_bizcocho marmol rabanado sweet ps_0.45</t>
+          <t>unknown_galleta maizena renata_0.36</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -6472,11 +6589,11 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Bizcocho Marmol Rabanado Sweet Ps</t>
+          <t>Galleta Maizena Renata</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>6.02</v>
+        <v>2.06</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -6493,12 +6610,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>unknown_bizcocho pudin de mantequilla y canela rebanao sweet ps_0.45</t>
+          <t>unknown_galleta manteca mocano_unknown</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -6511,11 +6628,11 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Bizcocho Pudin De Mantequilla Y Canela Rebanao Sweet Ps</t>
+          <t>Galleta Manteca Mocano</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>6.02</v>
+        <v>1.74</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -6532,12 +6649,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>unknown_capacillos desechables para hornear cupcakes colores mixtos over the top_unknown</t>
+          <t>unknown_galleta pozuelo chiky chocolate_unknown</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -6550,11 +6667,11 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Capacillos Desechables Para Hornear Cupcakes Colores Mixtos Over The Top</t>
+          <t>Galleta Pozuelo Chiky Chocolate</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>4.44</v>
+        <v>3.58</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -6571,12 +6688,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>unknown_capacillos grandes desechables para hornear cupcakes over the top_unknown</t>
+          <t>unknown_galleta pozuelo cremas chocolate_unknown</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -6589,11 +6706,11 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Capacillos Grandes Desechables Para Hornear Cupcakes Over The Top</t>
+          <t>Galleta Pozuelo Cremas Chocolate</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>2.22</v>
+        <v>1.88</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -6610,12 +6727,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>unknown_capacillos para mini cupcakes over the top_unknown</t>
+          <t>unknown_galleta pozuelo cremas fresa_unknown</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -6628,11 +6745,11 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Capacillos Para Mini Cupcakes Over The Top</t>
+          <t>Galleta Pozuelo Cremas Fresa</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>1.74</v>
+        <v>1.88</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -6649,12 +6766,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>unknown_galleta integral con ajonjoli gri gri_unknown</t>
+          <t>unknown_galleta pozuelo vainilla chocolate_0.3</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -6667,7 +6784,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Galleta Integral Con Ajonjoli Gri Gri</t>
+          <t>Galleta Pozuelo Vainilla Chocolate</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -6688,12 +6805,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>unknown_pan integral de centeno con semillas de calabaza mestemacher_0.5</t>
+          <t>unknown_galleta renata wafer choc_0.12</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -6706,11 +6823,11 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Pan Integral De Centeno Con Semillas De Calabaza Mestemacher</t>
+          <t>Galleta Renata Wafer Choc</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>2.85</v>
+        <v>0.95</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -6727,12 +6844,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>unknown_pan integral de centeno con semillas de girasol mestemacher_0.5</t>
+          <t>unknown_helado helados bon bizcocho_0.52</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -6745,11 +6862,11 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Pan Integral De Centeno Con Semillas De Girasol Mestemacher</t>
+          <t>Helado Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2.85</v>
+        <v>5.78</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -6766,12 +6883,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de vainilla spongy_0.15</t>
+          <t>unknown_helados bon bizcocho_0.26</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -6784,11 +6901,11 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1.17</v>
+        <v>3.71</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -6805,12 +6922,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>unknown_cup cake de vainilla con chispas sweet ps_0.28</t>
+          <t>unknown_mezcla para bizcocho renata coco_0.4</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -6823,11 +6940,11 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Cup Cake De Vainilla Con Chispas Sweet Ps</t>
+          <t>Mezcla Para Bizcocho Renata Coco</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>5.05</v>
+        <v>2.14</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -6844,12 +6961,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>unknown_galleta de avena vegan repeat_0.04</t>
+          <t>unknown_mezcla para bizcocho renata limon_0.4</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -6862,11 +6979,11 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Galleta De Avena Vegan Repeat</t>
+          <t>Mezcla Para Bizcocho Renata Limon</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>2.12</v>
+        <v>2.14</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -6883,12 +7000,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>unknown_galleta de avena vegan repeat_0.1</t>
+          <t>unknown_mezcla para bizcocho renata maiz_0.4</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -6901,11 +7018,11 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Galleta De Avena Vegan Repeat</t>
+          <t>Mezcla Para Bizcocho Renata Maiz</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>4.74</v>
+        <v>2.14</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -6922,12 +7039,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>unknown_galleta de chocolate chip artesanal green is my thing_unknown</t>
+          <t>unknown_mezcla para bizcocho renata naranja_0.4</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -6940,11 +7057,11 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Artesanal Green Is My Thing</t>
+          <t>Mezcla Para Bizcocho Renata Naranja</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>3.55</v>
+        <v>2.14</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -6961,12 +7078,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>unknown_galleta de chocolate chip vegana dbl_0.07</t>
+          <t>unknown_mezcla para bizcocho renata pina_0.4</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -6979,11 +7096,11 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Vegana Dbl</t>
+          <t>Mezcla Para Bizcocho Renata Pina</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>3.39</v>
+        <v>2.14</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -7000,12 +7117,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>unknown_galleta de chocolate chip vegana dbl_0.34</t>
+          <t>unknown_mezcla para bizcocho renata vainilla_0.4</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -7018,11 +7135,11 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Vegana Dbl</t>
+          <t>Mezcla Para Bizcocho Renata Vainilla</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>6.4</v>
+        <v>2.14</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -7039,12 +7156,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Carrefour</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>unknown_galleta integral con ajonjoli gri gri_unknown</t>
+          <t>unknown_paleta bon de bizcocho_unknown</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -7057,11 +7174,11 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Galleta Integral Con Ajonjoli Gri Gri</t>
+          <t>Paleta Bon De Bizcocho</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>1.81</v>
+        <v>0.63</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -7078,12 +7195,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>unknown_galletas artesanales de avena green is my thing_unknown</t>
+          <t>unknown_galleta lago mini party cacao_0.12</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -7096,11 +7213,11 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Galletas Artesanales De Avena Green Is My Thing</t>
+          <t>Galleta Lago Mini Party Cacao</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>3.55</v>
+        <v>1.66</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -7117,12 +7234,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>unknown_galletas artesanales de vainilla y guayaba ita abu_unknown</t>
+          <t>unknown_galletas de chocolate muuu con crema sabor a vainilla_unknown</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -7135,11 +7252,11 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Galletas Artesanales De Vainilla Y Guayaba Ita Abu</t>
+          <t>Galletas De Chocolate Muuu Con Crema Sabor A Vainilla</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>2.44</v>
+        <v>2.69</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -7156,12 +7273,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>unknown_mini brownies sweet ps_0.3</t>
+          <t>unknown_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -7174,11 +7291,11 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Mini Brownies Sweet Ps</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>5.69</v>
+        <v>0.46</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -7195,12 +7312,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>unknown_mini muffins choco chips mandul_0.2</t>
+          <t>unknown_galletas sandwich chocolate choco wow 10 und_0.48</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
@@ -7213,11 +7330,11 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Mini Muffins Choco Chips Mandul</t>
+          <t>Galletas Sandwich Chocolate Choco Wow 10 Und</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>3.79</v>
+        <v>2.14</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -7234,12 +7351,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>unknown_mini muffins choco stars mandul_0.21</t>
+          <t>unknown_leche sabor bizcocho vaquita rica uht_unknown</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -7252,11 +7369,11 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Mini Muffins Choco Stars Mandul</t>
+          <t>Leche Sabor Bizcocho Vaquita Rica Uht</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>3.79</v>
+        <v>0.48</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -7273,12 +7390,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Garrido</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>unknown_mini muffins rellenos de fresa mandul_0.21</t>
+          <t>unknown_mezcla para bizcocho de zanahoria supermoist_0.43</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -7291,11 +7408,11 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Mini Muffins Rellenos De Fresa Mandul</t>
+          <t>Mezcla Para Bizcocho De Zanahoria Supermoist</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>3.79</v>
+        <v>4.99</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -7312,12 +7429,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Jumbo</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>unknown_pan brioche chocolatechip bgourmet_0.4</t>
+          <t>unknown_barra de proteina sabor brownie de chocolate quest_0.06</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
@@ -7330,11 +7447,11 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Pan Brioche Chocolatechip Bgourmet</t>
+          <t>Barra De Proteina Sabor Brownie De Chocolate Quest</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>5.85</v>
+        <v>4.72</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -7351,12 +7468,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Merca Jumbo</t>
+          <t>Jumbo</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>unknown_pan brioche lonjeado bgourmet_0.5</t>
+          <t>unknown_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -7369,11 +7486,11 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Pan Brioche Lonjeado Bgourmet</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>6.85</v>
+        <v>0.47</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -7390,12 +7507,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>lu_galleta de chocolate chips sin ecovida_0.15</t>
+          <t>unknown_barra de proteina sabor brownie de chocolate quest_0.06</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
@@ -7403,16 +7520,16 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chips Sin Gluten Ecovida</t>
+          <t>Barra De Proteina Sabor Brownie De Chocolate Quest</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>3.72</v>
+        <v>4.71</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -7429,12 +7546,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de guineo rebanado sweet ps_0.45</t>
+          <t>unknown_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -7447,11 +7564,11 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Bizcocho De Guineo Rebanado Sweet Ps</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>6.02</v>
+        <v>0.46</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
@@ -7468,12 +7585,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de limon rebanado sweet ps_0.45</t>
+          <t>unknown_galletas sandwich chocolate choco wow 10 und_0.48</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -7486,11 +7603,11 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Bizcocho De Limon Rebanado Sweet Ps</t>
+          <t>Galletas Sandwich Chocolate Choco Wow 10 Und</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>6.02</v>
+        <v>2.2</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -7507,12 +7624,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de vainilla spongy_0.15</t>
+          <t>unknown_helado bizcocho bon 2 pintas_unknown</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -7525,11 +7642,11 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Helado Bizcocho Bon 2 Pintas</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>1.35</v>
+        <v>5.45</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -7546,12 +7663,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>unknown_bizcocho marmol rabanado sweet ps_0.45</t>
+          <t>unknown_helados bon bizcocho_0.26</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -7564,11 +7681,11 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Bizcocho Marmol Rabanado Sweet Ps</t>
+          <t>Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>6.02</v>
+        <v>3.69</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -7585,12 +7702,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Merca Jumbo</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>unknown_bizcocho pudin de mantequilla y canela rebanao sweet ps_0.45</t>
+          <t>unknown_tortillas chips kettle corn popcorners_0.14</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -7603,11 +7720,11 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Bizcocho Pudin De Mantequilla Y Canela Rebanao Sweet Ps</t>
+          <t>Tortillas Chips Kettle Corn Popcorners</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>6.02</v>
+        <v>3.63</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -7629,7 +7746,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>unknown_capacillos desechables para hornear cupcakes colores mixtos over the top_unknown</t>
+          <t>unknown_bagel crisps plain new york style_0.2</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -7642,11 +7759,11 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Capacillos Desechables Para Hornear Cupcakes Colores Mixtos Over The Top</t>
+          <t>Bagel Crisps Plain New York Style</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>4.44</v>
+        <v>3.56</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -7668,7 +7785,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>unknown_capacillos grandes desechables para hornear cupcakes over the top_unknown</t>
+          <t>unknown_bagel crisps sea salt new york style_0.2</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -7681,11 +7798,11 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Capacillos Grandes Desechables Para Hornear Cupcakes Over The Top</t>
+          <t>Bagel Crisps Sea Salt New York Style</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>2.22</v>
+        <v>3.56</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -7707,7 +7824,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>unknown_cup cake de vainilla con chispas sweet ps_0.28</t>
+          <t>unknown_barra de proteina sabor brownie de chocolate quest_0.06</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -7720,11 +7837,11 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Cup Cake De Vainilla Con Chispas Sweet Ps</t>
+          <t>Barra De Proteina Sabor Brownie De Chocolate Quest</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>5.07</v>
+        <v>4.72</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -7746,7 +7863,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>unknown_galleta de avena vegan repeat_0.04</t>
+          <t>unknown_galleta de mantequilla lotus_0.25</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -7759,11 +7876,11 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Galleta De Avena Vegan Repeat</t>
+          <t>Galleta De Mantequilla Lotus</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>2.14</v>
+        <v>4.28</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -7785,7 +7902,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>unknown_galleta de avena vegan repeat_0.1</t>
+          <t>unknown_galleta de mantequilla rellena de chocolate lotus_0.15</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -7798,11 +7915,11 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Galleta De Avena Vegan Repeat</t>
+          <t>Galleta De Mantequilla Rellena De Chocolate Lotus</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>4.75</v>
+        <v>3.49</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -7824,7 +7941,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>unknown_galleta de chocolate chip artesanal green is my thing_unknown</t>
+          <t>unknown_galletas cookie n cream axa_0.14</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -7837,11 +7954,11 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Artesanal Green Is My Thing</t>
+          <t>Galletas Cookie N Cream Axa</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>3.56</v>
+        <v>4.69</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -7863,7 +7980,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>unknown_galleta de chocolate chip vegana dbl_0.07</t>
+          <t>unknown_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -7876,11 +7993,11 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Vegana Dbl</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>3.41</v>
+        <v>0.47</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -7902,7 +8019,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>unknown_galleta de chocolate chip vegana dbl_0.34</t>
+          <t>unknown_leche sabor bizcocho vaquita rica uht_unknown</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -7915,11 +8032,11 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Galleta De Chocolate Chip Vegana Dbl</t>
+          <t>Leche Sabor Bizcocho Vaquita Rica Uht</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>6.42</v>
+        <v>0.46</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -7941,7 +8058,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>unknown_galletas artesanales de avena green is my thing_unknown</t>
+          <t>unknown_mezcla para bizcocho de zanahoria supermoist_0.43</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -7954,11 +8071,11 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Galletas Artesanales De Avena Green Is My Thing</t>
+          <t>Mezcla Para Bizcocho De Zanahoria Supermoist</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>3.56</v>
+        <v>4.83</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -7980,7 +8097,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>unknown_galletas artesanales de vainilla y guayaba ita abu_unknown</t>
+          <t>unknown_tortillas chips kettle corn popcorners_0.14</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -7993,11 +8110,11 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Galletas Artesanales De Vainilla Y Guayaba Ita Abu</t>
+          <t>Tortillas Chips Kettle Corn Popcorners</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>2.46</v>
+        <v>3.64</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -8014,12 +8131,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>unknown_galletas brownie brittle chocolate chips sheila gs_0.14</t>
+          <t>unknown_barra de proteina sabor brownie de chocolate quest_0.06</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -8032,11 +8149,11 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Chocolate Chips Sheila Gs</t>
+          <t>Barra De Proteina Sabor Brownie De Chocolate Quest</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>4.75</v>
+        <v>4.72</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -8053,12 +8170,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>unknown_galletas brownie brittle dark chocolate sea salt sheila gs_0.14</t>
+          <t>unknown_galleta wafers lago poker con avellanas 5 und_0.22</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -8071,11 +8188,11 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Dark Chocolate Sea Salt Sheila Gs</t>
+          <t>Galleta Wafers Lago Poker Con Avellanas 5 Und</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>4.75</v>
+        <v>2.99</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -8092,12 +8209,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>unknown_galletas brownie brittle salted caramel sheila gs_0.14</t>
+          <t>unknown_galleta wafers loacker sabor a coconut_0.04</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -8110,11 +8227,11 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Salted Caramel Sheila Gs</t>
+          <t>Galleta Wafers Loacker Sabor A Coconut</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>4.75</v>
+        <v>1.09</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -8131,12 +8248,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>unknown_galletas sin azucar rellenas de higo ecovida_0.15</t>
+          <t>unknown_galleta wafers loacker sabor a cremkakao_0.04</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -8149,11 +8266,11 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Galletas Sin Azucar Rellenas De Higo Ecovida</t>
+          <t>Galleta Wafers Loacker Sabor A Cremkakao</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>2.65</v>
+        <v>1.09</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -8170,12 +8287,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>unknown_mini brownies sweet ps_0.3</t>
+          <t>unknown_galleta wafers loacker sabor a napolitaner_0.04</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -8188,11 +8305,11 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Mini Brownies Sweet Ps</t>
+          <t>Galleta Wafers Loacker Sabor A Napolitaner</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>5.7</v>
+        <v>1.09</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -8209,12 +8326,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>unknown_mini cup cakes red velvet sweet ps_unknown</t>
+          <t>unknown_galleta wafers loacker sabor a vainilla_0.04</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -8227,11 +8344,11 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Mini Cup Cakes Red Velvet Sweet Ps</t>
+          <t>Galleta Wafers Loacker Sabor A Vainilla</t>
         </is>
       </c>
       <c r="I52" t="n">
-        <v>6.32</v>
+        <v>1.09</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -8248,12 +8365,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>unknown_mini muffins choco chips mandul_0.2</t>
+          <t>unknown_galletas cubanas dante con ajo_0.27</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -8266,11 +8383,11 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Mini Muffins Choco Chips Mandul</t>
+          <t>Galletas Cubanas Dante Con Ajo</t>
         </is>
       </c>
       <c r="I53" t="n">
-        <v>3.8</v>
+        <v>2.14</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -8287,12 +8404,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>unknown_mini muffins choco stars mandul_0.21</t>
+          <t>unknown_galletas cubanas dante_0.27</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -8305,11 +8422,11 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Mini Muffins Choco Stars Mandul</t>
+          <t>Galletas Cubanas Dante</t>
         </is>
       </c>
       <c r="I54" t="n">
-        <v>3.8</v>
+        <v>2.14</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -8326,12 +8443,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>unknown_mini muffins rellenos de fresa mandul_0.21</t>
+          <t>unknown_galletas de chocolate muuu con crema sabor a vainilla_unknown</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -8344,11 +8461,11 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Mini Muffins Rellenos De Fresa Mandul</t>
+          <t>Galletas De Chocolate Muuu Con Crema Sabor A Vainilla</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>3.8</v>
+        <v>2.76</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -8365,12 +8482,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>unknown_pan brioche chocolatechip bgourmet_0.4</t>
+          <t>unknown_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -8383,11 +8500,11 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Pan Brioche Chocolatechip Bgourmet</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="I56" t="n">
-        <v>5.86</v>
+        <v>0.48</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
@@ -8404,12 +8521,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>unknown_pan brioche lonjeado bgourmet_0.5</t>
+          <t>unknown_helado bon de bizcocho_0.52</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -8422,11 +8539,11 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Pan Brioche Lonjeado Bgourmet</t>
+          <t>Helado Bon De Bizcocho</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>6.86</v>
+        <v>6.32</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -8443,12 +8560,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>unknown_pan integral de centeno con semillas de calabaza mestemacher_0.5</t>
+          <t>unknown_helados bon bizcocho_0.26</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -8461,11 +8578,11 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Pan Integral De Centeno Con Semillas De Calabaza Mestemacher</t>
+          <t>Helados Bon Bizcocho</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>2.85</v>
+        <v>4.26</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -8482,12 +8599,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Plaza Lama</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>unknown_pan integral de centeno con semillas de girasol mestemacher_0.5</t>
+          <t>unknown_paleta bon de bizcocho_unknown</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -8500,11 +8617,11 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Pan Integral De Centeno Con Semillas De Girasol Mestemacher</t>
+          <t>Paleta Bon De Bizcocho</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>2.85</v>
+        <v>0.71</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
@@ -8526,7 +8643,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de vainilla spongy_0.15</t>
+          <t>unknown_tortillas chips kettle corn popcorners_0.14</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -8539,11 +8656,11 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Tortillas Chips Kettle Corn Popcorners</t>
         </is>
       </c>
       <c r="I60" t="n">
-        <v>1.35</v>
+        <v>3.64</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -8560,12 +8677,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Plaza Lama</t>
+          <t>Sirena</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>unknown_bizcocho spongy vainilla_0.23</t>
+          <t>unknown_galleta de mantequilla jules destrooper_0.1</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -8578,11 +8695,11 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Bizcocho Spongy Vainilla</t>
+          <t>Galleta De Mantequilla Jules Destrooper</t>
         </is>
       </c>
       <c r="I61" t="n">
-        <v>1.35</v>
+        <v>3.96</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
@@ -8599,12 +8716,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Ritmo</t>
+          <t>Sirena</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>unknown_bizcocho de vainilla spongy_0.15</t>
+          <t>unknown_galleta de mantequilla lotus_0.25</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -8617,11 +8734,11 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Bizcocho De Vainilla Spongy</t>
+          <t>Galleta De Mantequilla Lotus</t>
         </is>
       </c>
       <c r="I62" t="n">
-        <v>1.09</v>
+        <v>4.28</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
@@ -8643,7 +8760,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>lu_galleta ecovida sin coco_0.15</t>
+          <t>unknown_galleta lago mini party cacao_0.12</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -8651,16 +8768,16 @@
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Galleta Ecovida Sin Gluten Coco</t>
+          <t>Galleta Lago Mini Party Cacao</t>
         </is>
       </c>
       <c r="I63" t="n">
-        <v>3.72</v>
+        <v>2.06</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -8682,7 +8799,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>lu_galleta sin berrie ecovida_0.15</t>
+          <t>unknown_galleta snapd doble cheddar cheez it_0.21</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -8690,16 +8807,16 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>LU</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>Galleta Sin Gluten Berrie Ecovida</t>
+          <t>Galleta Snapd Doble Cheddar Cheez It</t>
         </is>
       </c>
       <c r="I64" t="n">
-        <v>3.72</v>
+        <v>4.6</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -8721,7 +8838,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>unknown_galletas brownie brittle chocolate chips sheila gs_0.14</t>
+          <t>unknown_galleta wafers lago wafers mini party avellanas_0.12</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -8734,11 +8851,11 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Chocolate Chips Sheila Gs</t>
+          <t>Galleta Wafers Lago Wafers Mini Party Avellanas</t>
         </is>
       </c>
       <c r="I65" t="n">
-        <v>5.15</v>
+        <v>2.06</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
@@ -8760,7 +8877,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>unknown_galletas brownie brittle dark chocolate sea salt sheila gs_0.14</t>
+          <t>unknown_galletas bridge wafer naranja_0.3</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -8773,11 +8890,11 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Dark Chocolate Sea Salt Sheila Gs</t>
+          <t>Galletas Bridge Wafer Naranja</t>
         </is>
       </c>
       <c r="I66" t="n">
-        <v>5.15</v>
+        <v>1.51</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
@@ -8799,7 +8916,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>unknown_galletas brownie brittle salted caramel sheila gs_0.14</t>
+          <t>unknown_galletas de chocolate y malvavisco mamut_0.03</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -8812,11 +8929,11 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Galletas Brownie Brittle Salted Caramel Sheila Gs</t>
+          <t>Galletas De Chocolate Y Malvavisco Mamut</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>5.15</v>
+        <v>0.48</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
@@ -8824,6 +8941,123 @@
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Dominican Republic</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Sirena</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>unknown_galletas sandwich chocolate choco wow 10 und_0.48</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Galletas Sandwich Chocolate Choco Wow 10 Und</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>right_only</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Dominican Republic</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Sirena</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>unknown_tortillas chips kettle corn popcorners_0.14</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Tortillas Chips Kettle Corn Popcorners</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>right_only</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Guyana</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Massy Stores Guyana</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>unknown_cheez it original 1 5oz_0.04</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Cheez-It Original  1.5oz</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>1.201923076923077</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>right_only</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>